<commit_message>
Group search score file by region only
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RzXUNWe52FPe7pzHpD5YVj
</commit_message>
<xml_diff>
--- a/Search_Score_Total_SoV_Jul1_Oct17_YTD_sorted.xlsx
+++ b/Search_Score_Total_SoV_Jul1_Oct17_YTD_sorted.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>Currys</t>
+          <t>Argos</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -569,10 +569,10 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>0.7817000000000001</v>
+        <v>0.6951000000000001</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>0.7554999999999999</v>
+        <v>0.6726000000000001</v>
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1" s="16">
@@ -593,10 +593,10 @@
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>0.6801999999999999</v>
+        <v>0.3129</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>0.6101</v>
+        <v>0.2939</v>
       </c>
     </row>
     <row r="5" ht="16.5" customHeight="1" s="16">
@@ -612,7 +612,7 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>Argos</t>
+          <t>Currys</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>0.6951000000000001</v>
+        <v>0.7817000000000001</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>0.6726000000000001</v>
+        <v>0.7554999999999999</v>
       </c>
     </row>
     <row r="6" ht="16.5" customHeight="1" s="16">
@@ -645,10 +645,10 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>0.3129</v>
+        <v>0.6801999999999999</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>0.2939</v>
+        <v>0.6101</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" s="16">
@@ -711,12 +711,12 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>FNAC-FR</t>
+          <t>EE-Store-GB</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -725,10 +725,10 @@
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>0.5103</v>
+        <v>0</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>0.5493</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1" s="16">
@@ -739,7 +739,7 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="C10" s="17" t="n"/>
@@ -749,10 +749,10 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>0.3395</v>
+        <v>0</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>0.3327000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1" s="16">
@@ -763,12 +763,12 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>Elkjop-NO</t>
+          <t>Media-Markt-DE</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -777,10 +777,10 @@
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>0.3948</v>
+        <v>0.3534</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>0.111</v>
+        <v>0.2716</v>
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1" s="16">
@@ -791,7 +791,7 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="C12" s="17" t="n"/>
@@ -801,10 +801,10 @@
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>0.1046</v>
+        <v>0.2783</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>0.0926</v>
+        <v>0.1972</v>
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1" s="16">
@@ -815,12 +815,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Media-Markt-DE</t>
+          <t>FNAC-FR</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -829,10 +829,10 @@
         </is>
       </c>
       <c r="E13" s="11" t="n">
-        <v>0.3534</v>
+        <v>0.5103</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>0.2716</v>
+        <v>0.5493</v>
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" s="16">
@@ -843,7 +843,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C14" s="17" t="n"/>
@@ -853,10 +853,10 @@
         </is>
       </c>
       <c r="E14" s="11" t="n">
-        <v>0.2783</v>
+        <v>0.3395</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>0.1972</v>
+        <v>0.3327000000000001</v>
       </c>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="16">
@@ -867,12 +867,12 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>EE-Store-GB</t>
+          <t>Elkjop-NO</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -881,10 +881,10 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>0</v>
+        <v>0.3948</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>0</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="16">
@@ -895,7 +895,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="C16" s="17" t="n"/>
@@ -905,10 +905,10 @@
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>0</v>
+        <v>0.1046</v>
       </c>
       <c r="F16" s="11" t="n">
-        <v>0</v>
+        <v>0.0926</v>
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="16">
@@ -954,7 +954,7 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>BestBuy-APP-US</t>
+          <t>BestBuy-US</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -963,10 +963,10 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>0.7873</v>
+        <v>0.7601</v>
       </c>
       <c r="F18" s="11" t="n">
-        <v>0.7873</v>
+        <v>0.8315</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="16">
@@ -987,10 +987,10 @@
         </is>
       </c>
       <c r="E19" s="11" t="n">
-        <v>0.4797</v>
+        <v>0.6327</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>0.4797</v>
+        <v>0.6368</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="16">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>BestBuy-US</t>
+          <t>Amazon-US</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -1015,10 +1015,10 @@
         </is>
       </c>
       <c r="E20" s="11" t="n">
-        <v>0.7601</v>
+        <v>0.4897</v>
       </c>
       <c r="F20" s="11" t="n">
-        <v>0.8315</v>
+        <v>0.5407999999999999</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" s="16">
@@ -1039,10 +1039,10 @@
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>0.6327</v>
+        <v>0.4776</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>0.6368</v>
+        <v>0.4727</v>
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1" s="16">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Target-APP-US</t>
+          <t>Walmart-US</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -1067,10 +1067,10 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>0.7356999999999999</v>
+        <v>0.5318999999999999</v>
       </c>
       <c r="F22" s="11" t="n">
-        <v>0.7356999999999999</v>
+        <v>0.5323</v>
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1" s="16">
@@ -1091,10 +1091,10 @@
         </is>
       </c>
       <c r="E23" s="11" t="n">
-        <v>0.2794</v>
+        <v>0.5435</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>0.2794</v>
+        <v>0.5757</v>
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1" s="16">
@@ -1209,12 +1209,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>BestBuy-CA</t>
+          <t>Amazon-APP-US</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1223,10 +1223,10 @@
         </is>
       </c>
       <c r="E28" s="11" t="n">
-        <v>0.5839</v>
+        <v>0.4209000000000001</v>
       </c>
       <c r="F28" s="11" t="n">
-        <v>0.6054999999999999</v>
+        <v>0.4209000000000001</v>
       </c>
     </row>
     <row r="29" ht="16.5" customHeight="1" s="16">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C29" s="17" t="n"/>
@@ -1247,10 +1247,10 @@
         </is>
       </c>
       <c r="E29" s="11" t="n">
-        <v>0.5435</v>
+        <v>0.4758</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>0.4523</v>
+        <v>0.4758</v>
       </c>
     </row>
     <row r="30" ht="16.5" customHeight="1" s="16">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Walmart-US</t>
+          <t>BestBuy-APP-US</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -1275,10 +1275,10 @@
         </is>
       </c>
       <c r="E30" s="11" t="n">
-        <v>0.5318999999999999</v>
+        <v>0.7873</v>
       </c>
       <c r="F30" s="11" t="n">
-        <v>0.5323</v>
+        <v>0.7873</v>
       </c>
     </row>
     <row r="31" ht="16.5" customHeight="1" s="16">
@@ -1299,10 +1299,10 @@
         </is>
       </c>
       <c r="E31" s="11" t="n">
-        <v>0.5435</v>
+        <v>0.4797</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>0.5757</v>
+        <v>0.4797</v>
       </c>
     </row>
     <row r="32" ht="16.5" customHeight="1" s="16">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Amazon-CA</t>
+          <t>Walmart-APP-US</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -1327,10 +1327,10 @@
         </is>
       </c>
       <c r="E32" s="11" t="n">
-        <v>0.5242</v>
+        <v>0.4958</v>
       </c>
       <c r="F32" s="11" t="n">
-        <v>0.5184000000000001</v>
+        <v>0.4958</v>
       </c>
     </row>
     <row r="33" ht="16.5" customHeight="1" s="16">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="C33" s="17" t="n"/>
@@ -1351,10 +1351,10 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>0.4705</v>
+        <v>0.5648</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>0.4425</v>
+        <v>0.5648</v>
       </c>
     </row>
     <row r="34" ht="16.5" customHeight="1" s="16">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>Walmart-APP-US</t>
+          <t>Target-APP-US</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -1379,10 +1379,10 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>0.4958</v>
+        <v>0.7356999999999999</v>
       </c>
       <c r="F34" s="11" t="n">
-        <v>0.4958</v>
+        <v>0.7356999999999999</v>
       </c>
     </row>
     <row r="35" ht="16.5" customHeight="1" s="16">
@@ -1403,10 +1403,10 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>0.5648</v>
+        <v>0.2794</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>0.5648</v>
+        <v>0.2794</v>
       </c>
     </row>
     <row r="36" ht="16.5" customHeight="1" s="16">
@@ -1417,12 +1417,12 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>Amazon-US</t>
+          <t>Amazon-CA</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -1431,10 +1431,10 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>0.4897</v>
+        <v>0.5242</v>
       </c>
       <c r="F36" s="11" t="n">
-        <v>0.5407999999999999</v>
+        <v>0.5184000000000001</v>
       </c>
     </row>
     <row r="37" ht="16.5" customHeight="1" s="16">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C37" s="17" t="n"/>
@@ -1455,10 +1455,10 @@
         </is>
       </c>
       <c r="E37" s="11" t="n">
-        <v>0.4776</v>
+        <v>0.4705</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>0.4727</v>
+        <v>0.4425</v>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="16">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>Walmart-EN-CA</t>
+          <t>BestBuy-CA</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -1483,10 +1483,10 @@
         </is>
       </c>
       <c r="E38" s="11" t="n">
-        <v>0.4643</v>
+        <v>0.5839</v>
       </c>
       <c r="F38" s="11" t="n">
-        <v>0.3472</v>
+        <v>0.6054999999999999</v>
       </c>
     </row>
     <row r="39" ht="16.5" customHeight="1" s="16">
@@ -1507,10 +1507,10 @@
         </is>
       </c>
       <c r="E39" s="11" t="n">
-        <v>0.5949</v>
+        <v>0.5435</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>0.5274</v>
+        <v>0.4523</v>
       </c>
     </row>
     <row r="40" ht="16.5" customHeight="1" s="16">
@@ -1521,12 +1521,12 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>Amazon-APP-US</t>
+          <t>Walmart-EN-CA</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -1535,10 +1535,10 @@
         </is>
       </c>
       <c r="E40" s="11" t="n">
-        <v>0.4209000000000001</v>
+        <v>0.4643</v>
       </c>
       <c r="F40" s="11" t="n">
-        <v>0.4209000000000001</v>
+        <v>0.3472</v>
       </c>
     </row>
     <row r="41" ht="16.5" customHeight="1" s="16">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C41" s="17" t="n"/>
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="E41" s="11" t="n">
-        <v>0.4758</v>
+        <v>0.5949</v>
       </c>
       <c r="F41" s="11" t="n">
-        <v>0.4758</v>
+        <v>0.5274</v>
       </c>
     </row>
     <row r="42" ht="16.5" customHeight="1" s="16">
@@ -1677,12 +1677,12 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>Amazon-IN</t>
+          <t>Telestra-AU</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -1691,10 +1691,10 @@
         </is>
       </c>
       <c r="E46" s="11" t="n">
-        <v>0.2808</v>
+        <v>0.2487</v>
       </c>
       <c r="F46" s="11" t="n">
-        <v>0.25</v>
+        <v>0.2487</v>
       </c>
     </row>
     <row r="47" ht="16.5" customHeight="1" s="16">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>AU</t>
         </is>
       </c>
       <c r="C47" s="17" t="n"/>
@@ -1715,10 +1715,10 @@
         </is>
       </c>
       <c r="E47" s="11" t="n">
-        <v>0.09449999999999999</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="F47" s="11" t="n">
-        <v>0.1</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="48" ht="16.5" customHeight="1" s="16">
@@ -1729,12 +1729,12 @@
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C48" s="14" t="inlineStr">
         <is>
-          <t>Telestra-AU</t>
+          <t>Amazon-JP</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
@@ -1743,10 +1743,10 @@
         </is>
       </c>
       <c r="E48" s="11" t="n">
-        <v>0.2487</v>
+        <v>0.1274</v>
       </c>
       <c r="F48" s="11" t="n">
-        <v>0.2487</v>
+        <v>0.2197</v>
       </c>
     </row>
     <row r="49" ht="16.5" customHeight="1" s="16">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>AU</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="C49" s="17" t="n"/>
@@ -1767,10 +1767,10 @@
         </is>
       </c>
       <c r="E49" s="11" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0248</v>
       </c>
       <c r="F49" s="11" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0238</v>
       </c>
     </row>
     <row r="50" ht="16.5" customHeight="1" s="16">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="C52" s="14" t="inlineStr">
         <is>
-          <t>Amazon-JP</t>
+          <t>BIC-JP</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -1847,10 +1847,10 @@
         </is>
       </c>
       <c r="E52" s="11" t="n">
-        <v>0.1274</v>
+        <v>0.07870000000000001</v>
       </c>
       <c r="F52" s="11" t="n">
-        <v>0.2197</v>
+        <v>0.08220000000000001</v>
       </c>
     </row>
     <row r="53" ht="16.5" customHeight="1" s="16">
@@ -1871,10 +1871,10 @@
         </is>
       </c>
       <c r="E53" s="11" t="n">
-        <v>0.0248</v>
+        <v>0.0144</v>
       </c>
       <c r="F53" s="11" t="n">
-        <v>0.0238</v>
+        <v>0.0363</v>
       </c>
     </row>
     <row r="54" ht="16.5" customHeight="1" s="16">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="C54" s="14" t="inlineStr">
         <is>
-          <t>Flipkart-APP-IN</t>
+          <t>Amazon-IN</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -1899,10 +1899,10 @@
         </is>
       </c>
       <c r="E54" s="11" t="n">
-        <v>0.1177</v>
+        <v>0.2808</v>
       </c>
       <c r="F54" s="11" t="n">
-        <v>0.1177</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="55" ht="16.5" customHeight="1" s="16">
@@ -1923,10 +1923,10 @@
         </is>
       </c>
       <c r="E55" s="11" t="n">
-        <v>0.2323</v>
+        <v>0.09449999999999999</v>
       </c>
       <c r="F55" s="11" t="n">
-        <v>0.2323</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="56" ht="16.5" customHeight="1" s="16">
@@ -1989,12 +1989,12 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
-          <t>BIC-JP</t>
+          <t>Flipkart-APP-IN</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -2003,10 +2003,10 @@
         </is>
       </c>
       <c r="E58" s="11" t="n">
-        <v>0.07870000000000001</v>
+        <v>0.1177</v>
       </c>
       <c r="F58" s="11" t="n">
-        <v>0.08220000000000001</v>
+        <v>0.1177</v>
       </c>
     </row>
     <row r="59" ht="16.5" customHeight="1" s="16">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C59" s="17" t="n"/>
@@ -2027,10 +2027,10 @@
         </is>
       </c>
       <c r="E59" s="11" t="n">
-        <v>0.0144</v>
+        <v>0.2323</v>
       </c>
       <c r="F59" s="11" t="n">
-        <v>0.0363</v>
+        <v>0.2323</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="16"/>

</xml_diff>